<commit_message>
updated some transformations in data processing
</commit_message>
<xml_diff>
--- a/data_processing/transformations/templates/calibrated/uganda/model_input_variables_uganda_se_calibrated.xlsx
+++ b/data_processing/transformations/templates/calibrated/uganda/model_input_variables_uganda_se_calibrated.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="78">
   <si>
     <t>subsector</t>
   </si>
@@ -42,6 +42,174 @@
   </si>
   <si>
     <t>min_55</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>28</t>
+  </si>
+  <si>
+    <t>29</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>31</t>
+  </si>
+  <si>
+    <t>32</t>
+  </si>
+  <si>
+    <t>33</t>
+  </si>
+  <si>
+    <t>34</t>
+  </si>
+  <si>
+    <t>35</t>
+  </si>
+  <si>
+    <t>36</t>
+  </si>
+  <si>
+    <t>37</t>
+  </si>
+  <si>
+    <t>38</t>
+  </si>
+  <si>
+    <t>39</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>41</t>
+  </si>
+  <si>
+    <t>42</t>
+  </si>
+  <si>
+    <t>43</t>
+  </si>
+  <si>
+    <t>44</t>
+  </si>
+  <si>
+    <t>45</t>
+  </si>
+  <si>
+    <t>46</t>
+  </si>
+  <si>
+    <t>47</t>
+  </si>
+  <si>
+    <t>48</t>
+  </si>
+  <si>
+    <t>49</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>51</t>
+  </si>
+  <si>
+    <t>52</t>
+  </si>
+  <si>
+    <t>53</t>
+  </si>
+  <si>
+    <t>54</t>
+  </si>
+  <si>
+    <t>55</t>
   </si>
   <si>
     <t>Economy</t>
@@ -469,181 +637,181 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1">
-        <v>0</v>
-      </c>
-      <c r="K1" s="1">
-        <v>1</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2</v>
-      </c>
-      <c r="M1" s="1">
-        <v>3</v>
-      </c>
-      <c r="N1" s="1">
-        <v>4</v>
-      </c>
-      <c r="O1" s="1">
-        <v>5</v>
-      </c>
-      <c r="P1" s="1">
-        <v>6</v>
-      </c>
-      <c r="Q1" s="1">
-        <v>7</v>
-      </c>
-      <c r="R1" s="1">
-        <v>8</v>
-      </c>
-      <c r="S1" s="1">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="T1" s="1">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="U1" s="1">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="V1" s="1">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="W1" s="1">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="X1" s="1">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="Y1" s="1">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Z1" s="1">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="AA1" s="1">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="AB1" s="1">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="AC1" s="1">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="AD1" s="1">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="AE1" s="1">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="AF1" s="1">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="AG1" s="1">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="AH1" s="1">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="AI1" s="1">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AJ1" s="1">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="AK1" s="1">
+      <c r="AB1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="AL1" s="1">
+      <c r="AC1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="AM1" s="1">
+      <c r="AD1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="AN1" s="1">
+      <c r="AE1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="AO1" s="1">
+      <c r="AF1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="AP1" s="1">
+      <c r="AG1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="AQ1" s="1">
+      <c r="AH1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="AR1" s="1">
+      <c r="AI1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="AS1" s="1">
+      <c r="AJ1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="AT1" s="1">
+      <c r="AK1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AU1" s="1">
+      <c r="AL1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="AV1" s="1">
+      <c r="AM1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AW1" s="1">
+      <c r="AN1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="AX1" s="1">
+      <c r="AO1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="AY1" s="1">
+      <c r="AP1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="AZ1" s="1">
+      <c r="AQ1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="BA1" s="1">
+      <c r="AR1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="BB1" s="1">
+      <c r="AS1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="BC1" s="1">
+      <c r="AT1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="BD1" s="1">
+      <c r="AU1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="BE1" s="1">
+      <c r="AV1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="BF1" s="1">
+      <c r="AW1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="BG1" s="1">
+      <c r="AX1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="BH1" s="1">
+      <c r="AY1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="BI1" s="1">
+      <c r="AZ1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="BJ1" s="1">
+      <c r="BA1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="BK1" s="1">
+      <c r="BB1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="BL1" s="1">
+      <c r="BC1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="BM1" s="1">
+      <c r="BD1" s="1" t="s">
         <v>55</v>
+      </c>
+      <c r="BE1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="BF1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="BG1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="BH1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="BI1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="BJ1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="BK1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="BL1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="BM1" s="1" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:65">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>65</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>67</v>
       </c>
       <c r="H2">
         <v>1</v>
@@ -822,10 +990,10 @@
     </row>
     <row r="3" spans="1:65">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>66</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>68</v>
       </c>
       <c r="H3">
         <v>1</v>
@@ -1004,10 +1172,10 @@
     </row>
     <row r="4" spans="1:65">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>66</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>69</v>
       </c>
       <c r="H4">
         <v>1</v>
@@ -1186,10 +1354,10 @@
     </row>
     <row r="5" spans="1:65">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>66</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>70</v>
       </c>
       <c r="H5">
         <v>1</v>
@@ -1368,10 +1536,10 @@
     </row>
     <row r="6" spans="1:65">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>66</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>71</v>
       </c>
       <c r="H6">
         <v>1</v>
@@ -1550,10 +1718,10 @@
     </row>
     <row r="7" spans="1:65">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>66</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>72</v>
       </c>
       <c r="H7">
         <v>1</v>
@@ -1732,10 +1900,10 @@
     </row>
     <row r="8" spans="1:65">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>66</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>73</v>
       </c>
       <c r="H8">
         <v>1</v>
@@ -1914,10 +2082,10 @@
     </row>
     <row r="9" spans="1:65">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>66</v>
       </c>
       <c r="B9" t="s">
-        <v>18</v>
+        <v>74</v>
       </c>
       <c r="H9">
         <v>1</v>
@@ -2096,10 +2264,10 @@
     </row>
     <row r="10" spans="1:65">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>66</v>
       </c>
       <c r="B10" t="s">
-        <v>19</v>
+        <v>75</v>
       </c>
       <c r="H10">
         <v>1</v>
@@ -2278,10 +2446,10 @@
     </row>
     <row r="11" spans="1:65">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>66</v>
       </c>
       <c r="B11" t="s">
-        <v>20</v>
+        <v>76</v>
       </c>
       <c r="H11">
         <v>1</v>
@@ -2460,10 +2628,10 @@
     </row>
     <row r="12" spans="1:65">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>66</v>
       </c>
       <c r="B12" t="s">
-        <v>21</v>
+        <v>77</v>
       </c>
       <c r="H12">
         <v>1</v>
@@ -2678,181 +2846,181 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1">
-        <v>0</v>
-      </c>
-      <c r="K1" s="1">
-        <v>1</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2</v>
-      </c>
-      <c r="M1" s="1">
-        <v>3</v>
-      </c>
-      <c r="N1" s="1">
-        <v>4</v>
-      </c>
-      <c r="O1" s="1">
-        <v>5</v>
-      </c>
-      <c r="P1" s="1">
-        <v>6</v>
-      </c>
-      <c r="Q1" s="1">
-        <v>7</v>
-      </c>
-      <c r="R1" s="1">
-        <v>8</v>
-      </c>
-      <c r="S1" s="1">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="T1" s="1">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="U1" s="1">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="V1" s="1">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="W1" s="1">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="X1" s="1">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="Y1" s="1">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Z1" s="1">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="AA1" s="1">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="AB1" s="1">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="AC1" s="1">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="AD1" s="1">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="AE1" s="1">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="AF1" s="1">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="AG1" s="1">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="AH1" s="1">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="AI1" s="1">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AJ1" s="1">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="AK1" s="1">
+      <c r="AB1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="AL1" s="1">
+      <c r="AC1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="AM1" s="1">
+      <c r="AD1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="AN1" s="1">
+      <c r="AE1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="AO1" s="1">
+      <c r="AF1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="AP1" s="1">
+      <c r="AG1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="AQ1" s="1">
+      <c r="AH1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="AR1" s="1">
+      <c r="AI1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="AS1" s="1">
+      <c r="AJ1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="AT1" s="1">
+      <c r="AK1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AU1" s="1">
+      <c r="AL1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="AV1" s="1">
+      <c r="AM1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AW1" s="1">
+      <c r="AN1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="AX1" s="1">
+      <c r="AO1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="AY1" s="1">
+      <c r="AP1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="AZ1" s="1">
+      <c r="AQ1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="BA1" s="1">
+      <c r="AR1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="BB1" s="1">
+      <c r="AS1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="BC1" s="1">
+      <c r="AT1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="BD1" s="1">
+      <c r="AU1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="BE1" s="1">
+      <c r="AV1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="BF1" s="1">
+      <c r="AW1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="BG1" s="1">
+      <c r="AX1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="BH1" s="1">
+      <c r="AY1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="BI1" s="1">
+      <c r="AZ1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="BJ1" s="1">
+      <c r="BA1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="BK1" s="1">
+      <c r="BB1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="BL1" s="1">
+      <c r="BC1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="BM1" s="1">
+      <c r="BD1" s="1" t="s">
         <v>55</v>
+      </c>
+      <c r="BE1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="BF1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="BG1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="BH1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="BI1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="BJ1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="BK1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="BL1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="BM1" s="1" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:65">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>66</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>71</v>
       </c>
       <c r="H2">
         <v>1</v>

</xml_diff>

<commit_message>
updated a number of inputs and transformations
</commit_message>
<xml_diff>
--- a/data_processing/transformations/templates/calibrated/uganda/model_input_variables_uganda_se_calibrated.xlsx
+++ b/data_processing/transformations/templates/calibrated/uganda/model_input_variables_uganda_se_calibrated.xlsx
@@ -3068,130 +3068,130 @@
         <v>0.88</v>
       </c>
       <c r="W2">
-        <v>0.8613953488372093</v>
+        <v>0.8594285714285713</v>
       </c>
       <c r="X2">
-        <v>0.8432558139534885</v>
+        <v>0.8394285714285714</v>
       </c>
       <c r="Y2">
-        <v>0.8255813953488371</v>
+        <v>0.82</v>
       </c>
       <c r="Z2">
-        <v>0.8083720930232559</v>
+        <v>0.8011428571428572</v>
       </c>
       <c r="AA2">
-        <v>0.7916279069767441</v>
+        <v>0.7828571428571428</v>
       </c>
       <c r="AB2">
-        <v>0.7753488372093023</v>
+        <v>0.7651428571428571</v>
       </c>
       <c r="AC2">
-        <v>0.7595348837209303</v>
+        <v>0.7480000000000001</v>
       </c>
       <c r="AD2">
-        <v>0.7441860465116279</v>
+        <v>0.7314285714285715</v>
       </c>
       <c r="AE2">
-        <v>0.7293023255813953</v>
+        <v>0.7154285714285714</v>
       </c>
       <c r="AF2">
-        <v>0.7148837209302326</v>
+        <v>0.7</v>
       </c>
       <c r="AG2">
-        <v>0.7009302325581396</v>
+        <v>0.6851428571428572</v>
       </c>
       <c r="AH2">
-        <v>0.6874418604651162</v>
+        <v>0.6708571428571428</v>
       </c>
       <c r="AI2">
-        <v>0.6744186046511629</v>
+        <v>0.6571428571428571</v>
       </c>
       <c r="AJ2">
-        <v>0.6618604651162791</v>
+        <v>0.644</v>
       </c>
       <c r="AK2">
-        <v>0.6497674418604651</v>
+        <v>0.6314285714285713</v>
       </c>
       <c r="AL2">
-        <v>0.6381395348837209</v>
+        <v>0.6194285714285714</v>
       </c>
       <c r="AM2">
-        <v>0.6269767441860464</v>
+        <v>0.608</v>
       </c>
       <c r="AN2">
-        <v>0.6162790697674418</v>
+        <v>0.5971428571428572</v>
       </c>
       <c r="AO2">
-        <v>0.6116279069767442</v>
+        <v>0.5914285714285714</v>
       </c>
       <c r="AP2">
-        <v>0.6069767441860465</v>
+        <v>0.5857142857142856</v>
       </c>
       <c r="AQ2">
-        <v>0.6023255813953488</v>
+        <v>0.58</v>
       </c>
       <c r="AR2">
-        <v>0.5976744186046512</v>
+        <v>0.5742857142857143</v>
       </c>
       <c r="AS2">
-        <v>0.5930232558139534</v>
+        <v>0.5685714285714285</v>
       </c>
       <c r="AT2">
-        <v>0.5883720930232558</v>
+        <v>0.5628571428571428</v>
       </c>
       <c r="AU2">
-        <v>0.5837209302325581</v>
+        <v>0.5571428571428572</v>
       </c>
       <c r="AV2">
-        <v>0.5790697674418605</v>
+        <v>0.5514285714285714</v>
       </c>
       <c r="AW2">
-        <v>0.5744186046511628</v>
+        <v>0.5457142857142857</v>
       </c>
       <c r="AX2">
-        <v>0.5697674418604651</v>
+        <v>0.54</v>
       </c>
       <c r="AY2">
-        <v>0.5651162790697675</v>
+        <v>0.5342857142857143</v>
       </c>
       <c r="AZ2">
-        <v>0.5604651162790697</v>
+        <v>0.5285714285714286</v>
       </c>
       <c r="BA2">
-        <v>0.5558139534883721</v>
+        <v>0.5228571428571429</v>
       </c>
       <c r="BB2">
-        <v>0.5511627906976744</v>
+        <v>0.5171428571428571</v>
       </c>
       <c r="BC2">
-        <v>0.5465116279069767</v>
+        <v>0.5114285714285715</v>
       </c>
       <c r="BD2">
-        <v>0.5418604651162791</v>
+        <v>0.5057142857142857</v>
       </c>
       <c r="BE2">
-        <v>0.5372093023255814</v>
+        <v>0.5</v>
       </c>
       <c r="BF2">
-        <v>0.5325581395348837</v>
+        <v>0.5</v>
       </c>
       <c r="BG2">
-        <v>0.5279069767441861</v>
+        <v>0.5</v>
       </c>
       <c r="BH2">
-        <v>0.5232558139534884</v>
+        <v>0.5</v>
       </c>
       <c r="BI2">
-        <v>0.5186046511627908</v>
+        <v>0.5</v>
       </c>
       <c r="BJ2">
-        <v>0.513953488372093</v>
+        <v>0.5</v>
       </c>
       <c r="BK2">
-        <v>0.5093023255813953</v>
+        <v>0.5</v>
       </c>
       <c r="BL2">
-        <v>0.5046511627906977</v>
+        <v>0.5</v>
       </c>
       <c r="BM2">
         <v>0.5</v>

</xml_diff>

<commit_message>
Updated a number of inputs, including fertilizer and lime, and adjusted baseline to align better with inventory nomenclature
</commit_message>
<xml_diff>
--- a/data_processing/transformations/templates/calibrated/uganda/model_input_variables_uganda_se_calibrated.xlsx
+++ b/data_processing/transformations/templates/calibrated/uganda/model_input_variables_uganda_se_calibrated.xlsx
@@ -23,6 +23,9 @@
     <t>variable</t>
   </si>
   <si>
+    <t>variable_trajectory_group</t>
+  </si>
+  <si>
     <t>normalize_group</t>
   </si>
   <si>
@@ -30,9 +33,6 @@
   </si>
   <si>
     <t>uniform_scaling_q</t>
-  </si>
-  <si>
-    <t>variable_trajectory_group</t>
   </si>
   <si>
     <t>variable_trajectory_group_trajectory_type</t>
@@ -813,11 +813,14 @@
       <c r="B2" t="s">
         <v>67</v>
       </c>
+      <c r="C2">
+        <v>62</v>
+      </c>
       <c r="H2">
         <v>1</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="J2">
         <v>79.03</v>
@@ -1181,7 +1184,7 @@
         <v>1</v>
       </c>
       <c r="I4">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J4">
         <v>1</v>
@@ -1541,6 +1544,9 @@
       <c r="B6" t="s">
         <v>71</v>
       </c>
+      <c r="C6">
+        <v>29</v>
+      </c>
       <c r="H6">
         <v>1</v>
       </c>
@@ -2451,11 +2457,14 @@
       <c r="B11" t="s">
         <v>76</v>
       </c>
+      <c r="C11">
+        <v>65</v>
+      </c>
       <c r="H11">
-        <v>1</v>
+        <v>1.05</v>
       </c>
       <c r="I11">
-        <v>1</v>
+        <v>0.85</v>
       </c>
       <c r="J11">
         <v>27658870</v>
@@ -2633,11 +2642,14 @@
       <c r="B12" t="s">
         <v>77</v>
       </c>
+      <c r="C12">
+        <v>65</v>
+      </c>
       <c r="H12">
-        <v>1</v>
+        <v>1.05</v>
       </c>
       <c r="I12">
-        <v>1</v>
+        <v>0.85</v>
       </c>
       <c r="J12">
         <v>7933333</v>
@@ -3022,6 +3034,9 @@
       <c r="B2" t="s">
         <v>71</v>
       </c>
+      <c r="C2">
+        <v>29</v>
+      </c>
       <c r="H2">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
last commit before attempting to push biomass use further back
</commit_message>
<xml_diff>
--- a/data_processing/transformations/templates/calibrated/uganda/model_input_variables_uganda_se_calibrated.xlsx
+++ b/data_processing/transformations/templates/calibrated/uganda/model_input_variables_uganda_se_calibrated.xlsx
@@ -8,14 +8,15 @@
   </bookViews>
   <sheets>
     <sheet name="strategy_id-0" sheetId="1" r:id="rId1"/>
-    <sheet name="strategy_id-6004" sheetId="2" r:id="rId2"/>
+    <sheet name="strategy_id-6007" sheetId="2" r:id="rId2"/>
+    <sheet name="strategy_id-6063" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="78">
   <si>
     <t>subsector</t>
   </si>
@@ -814,7 +815,7 @@
         <v>67</v>
       </c>
       <c r="C2">
-        <v>59</v>
+        <v>36</v>
       </c>
       <c r="H2">
         <v>1</v>
@@ -1544,9 +1545,6 @@
       <c r="B6" t="s">
         <v>71</v>
       </c>
-      <c r="C6">
-        <v>27</v>
-      </c>
       <c r="H6">
         <v>1</v>
       </c>
@@ -2458,7 +2456,7 @@
         <v>76</v>
       </c>
       <c r="C11">
-        <v>62</v>
+        <v>39</v>
       </c>
       <c r="H11">
         <v>1.05</v>
@@ -2643,7 +2641,7 @@
         <v>77</v>
       </c>
       <c r="C12">
-        <v>62</v>
+        <v>39</v>
       </c>
       <c r="H12">
         <v>1.05</v>
@@ -3034,8 +3032,394 @@
       <c r="B2" t="s">
         <v>71</v>
       </c>
-      <c r="C2">
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
+      </c>
+      <c r="N2">
+        <v>1</v>
+      </c>
+      <c r="O2">
+        <v>1</v>
+      </c>
+      <c r="P2">
+        <v>1</v>
+      </c>
+      <c r="Q2">
+        <v>1</v>
+      </c>
+      <c r="R2">
+        <v>1</v>
+      </c>
+      <c r="S2">
+        <v>1</v>
+      </c>
+      <c r="T2">
+        <v>1</v>
+      </c>
+      <c r="U2">
+        <v>1</v>
+      </c>
+      <c r="V2">
+        <v>1</v>
+      </c>
+      <c r="W2">
+        <v>1</v>
+      </c>
+      <c r="X2">
+        <v>0.98</v>
+      </c>
+      <c r="Y2">
+        <v>0.96</v>
+      </c>
+      <c r="Z2">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="AA2">
+        <v>0.9199999999999999</v>
+      </c>
+      <c r="AB2">
+        <v>0.9</v>
+      </c>
+      <c r="AC2">
+        <v>0.8799999999999999</v>
+      </c>
+      <c r="AD2">
+        <v>0.8600000000000001</v>
+      </c>
+      <c r="AE2">
+        <v>0.8400000000000001</v>
+      </c>
+      <c r="AF2">
+        <v>0.8200000000000001</v>
+      </c>
+      <c r="AG2">
+        <v>0.8</v>
+      </c>
+      <c r="AH2">
+        <v>0.78</v>
+      </c>
+      <c r="AI2">
+        <v>0.76</v>
+      </c>
+      <c r="AJ2">
+        <v>0.74</v>
+      </c>
+      <c r="AK2">
+        <v>0.72</v>
+      </c>
+      <c r="AL2">
+        <v>0.7</v>
+      </c>
+      <c r="AM2">
+        <v>0.68</v>
+      </c>
+      <c r="AN2">
+        <v>0.6599999999999999</v>
+      </c>
+      <c r="AO2">
+        <v>0.64</v>
+      </c>
+      <c r="AP2">
+        <v>0.62</v>
+      </c>
+      <c r="AQ2">
+        <v>0.6</v>
+      </c>
+      <c r="AR2">
+        <v>0.5800000000000001</v>
+      </c>
+      <c r="AS2">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="AT2">
+        <v>0.54</v>
+      </c>
+      <c r="AU2">
+        <v>0.52</v>
+      </c>
+      <c r="AV2">
+        <v>0.5</v>
+      </c>
+      <c r="AW2">
+        <v>0.48</v>
+      </c>
+      <c r="AX2">
+        <v>0.46</v>
+      </c>
+      <c r="AY2">
+        <v>0.4399999999999999</v>
+      </c>
+      <c r="AZ2">
+        <v>0.4199999999999999</v>
+      </c>
+      <c r="BA2">
+        <v>0.4</v>
+      </c>
+      <c r="BB2">
+        <v>0.38</v>
+      </c>
+      <c r="BC2">
+        <v>0.36</v>
+      </c>
+      <c r="BD2">
+        <v>0.34</v>
+      </c>
+      <c r="BE2">
+        <v>0.32</v>
+      </c>
+      <c r="BF2">
+        <v>0.3</v>
+      </c>
+      <c r="BG2">
+        <v>0.3</v>
+      </c>
+      <c r="BH2">
+        <v>0.3</v>
+      </c>
+      <c r="BI2">
+        <v>0.3</v>
+      </c>
+      <c r="BJ2">
+        <v>0.3</v>
+      </c>
+      <c r="BK2">
+        <v>0.3</v>
+      </c>
+      <c r="BL2">
+        <v>0.3</v>
+      </c>
+      <c r="BM2">
+        <v>0.3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:BM2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:65">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="1" t="s">
         <v>27</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AL1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AM1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AO1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AQ1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AR1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AS1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AT1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AU1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="AV1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="AW1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AX1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="AY1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="AZ1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="BA1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="BB1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="BC1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="BD1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="BE1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="BF1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="BG1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="BH1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="BI1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="BJ1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="BK1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="BL1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="BM1" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="2" spans="1:65">
+      <c r="A2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" t="s">
+        <v>71</v>
       </c>
       <c r="H2">
         <v>1</v>

</xml_diff>